<commit_message>
Skip Other variant_category case-insensitively and cover the fixture's OTHER row
The v1 workbook gains an IGN / OTHER row. Match variant_category uppercased so any casing of 'Other' (and MUTATION/CNV/SV/SIGNATURE) is recognized rather than falling through to the unrecognized-value warning. Assert the OTHER row is retained in the normalized findings (lossless patient_data) but produces no clinical/genomic doc.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/test-pt-data-v1.0.0.xlsx
+++ b/tests/fixtures/test-pt-data-v1.0.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deemer/Documents/git-repos/ctm-report-preview/tests/fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F99F6F-EAAA-A244-A817-7728308CBEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{829DEAB9-7D70-D44F-8A02-E7A59BA7750B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-106940" yWindow="600" windowWidth="36540" windowHeight="21000" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-106940" yWindow="600" windowWidth="30220" windowHeight="21000" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="_legend" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="177">
   <si>
     <t>Column type</t>
   </si>
@@ -557,6 +557,12 @@
   </si>
   <si>
     <t>Stable</t>
+  </si>
+  <si>
+    <t>IGN</t>
+  </si>
+  <si>
+    <t>OTHER</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1087,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
@@ -1558,6 +1564,20 @@
       </c>
       <c r="D24" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" t="s">
+        <v>175</v>
+      </c>
+      <c r="D25" t="s">
+        <v>176</v>
       </c>
     </row>
   </sheetData>

</xml_diff>